<commit_message>
create a debug and also full experiement bat file for easier to run simulation and also update ipynb file for better labelling and running plot.
</commit_message>
<xml_diff>
--- a/data/figures/phase0/phase0_baseline_metrics.xlsx
+++ b/data/figures/phase0/phase0_baseline_metrics.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>mean_reachF</t>
   </si>
@@ -70,10 +70,16 @@
     <t>n_t_peak_r</t>
   </si>
   <si>
+    <t>cond</t>
+  </si>
+  <si>
     <t>Condition</t>
   </si>
   <si>
-    <t>Baseline</t>
+    <t>BL</t>
+  </si>
+  <si>
+    <t>bl</t>
   </si>
 </sst>
 </file>
@@ -431,12 +437,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -492,64 +498,70 @@
       <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="T1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:20">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2">
-        <v>62.34</v>
+        <v>62.653</v>
       </c>
       <c r="C2">
-        <v>7.068</v>
+        <v>7.006</v>
       </c>
       <c r="D2">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="E2">
         <v>99.997</v>
       </c>
       <c r="F2">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
       <c r="G2">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="H2">
-        <v>546.295</v>
+        <v>542.828</v>
       </c>
       <c r="I2">
-        <v>144.19</v>
+        <v>140.999</v>
       </c>
       <c r="J2">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="K2">
-        <v>2157.574</v>
+        <v>2154.305</v>
       </c>
       <c r="L2">
-        <v>30.883</v>
+        <v>31.588</v>
       </c>
       <c r="M2">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="N2">
-        <v>22.607</v>
+        <v>22.892</v>
       </c>
       <c r="O2">
-        <v>4.001</v>
+        <v>4.008</v>
       </c>
       <c r="P2">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="Q2">
-        <v>56.262</v>
+        <v>56.424</v>
       </c>
       <c r="R2">
-        <v>3.039</v>
+        <v>2.97</v>
       </c>
       <c r="S2">
-        <v>183</v>
+        <v>203</v>
+      </c>
+      <c r="T2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>